<commit_message>
chore: update news radar report 2026-10-15
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-10-14.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-10-14.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -477,12 +477,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Three Key Messages for Employers Managing Rising Healthcare Costs</t>
+          <t>Market Barriers Keep Biosimilars From Gaining Ground Against Brand-Name Rivals</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Healthcare expert Katie Martin outlines critical strategies for self-funded employers grappling with escalating medical and pharmacy benefit expenses. The guidance emphasizes actionable plan design and cost-management approaches that directly impact commercial employer health plans.</t>
+          <t>This Q&amp;A examines the persistent market and formulary barriers that prevent biosimilars from displacing high-cost brand-name biologics. For self-funded employers and PBMs, understanding these adoption hurdles is critical for unlocking potential specialty drug savings.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -492,12 +492,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 22:27:25 GMT</t>
+          <t>Wed, 14 Oct 2026 14:03:43 GMT</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxQbUtkSlBabWZvU09lMzEzOGhGbnhwMjNoRzdDaXZhRVNCZWNsd3BVaGZvd3A4ZUpWT2ozakZYc3g4R1NsM1I0ZVZ5MHhlR254cFFvYzc2V0hIWkl6OVhmUFh3RTJQZ3NEYlZQMmdac2RsbE5EMHlRdWpFYmFmdlNic3NROHFXY3pkNHZYa0laR3BKUnlhZHcxRXczS20wVWZZNGR6ZU91dGx5VGxVS3pNSnJRNGVXd28?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOMTEwSHlrSi0zN2ZsVDNldXdOYzc3MVhFRmpFanE1NVdpZlhON2pTdVVDZkdNSVZMT0l0c0w2MWFqak05dTY0NFh0a0phZXMxblNBQ1ZVSXFNODVuTy05YlJzUXZvaldNUXVuVVMyaWJqOG9SLVFZYk04b25NQzNnUWtaVFRkVy14U0h3eXJzN1dhTWxzMEhDT0V0ZWlRZkRWeVd4N1EyNDRvU2JPZDRKM0xaOGUwdkxkVndKb1JB?oc=5</t>
         </is>
       </c>
     </row>
@@ -507,27 +507,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>High Unit Prices Drive U.S. Employer Healthcare Spending</t>
+          <t>Study Shows Non-Responding Patients Continue GLP-1 Therapy Despite Lack of Efficacy</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Expert analysis underscores that underlying unit prices—rather than just utilization—remain the primary driver of escalating healthcare costs for U.S. employers. For self-funded plans, this highlights the critical need for aggressive price containment strategies within pharmacy and medical benefits. The discussion emphasizes that managing cost trends requires tackling unit prices directly rather than focusing solely on utilization management.</t>
+          <t>A new study reveals that many patients who fail to experience meaningful weight loss or glycemic control on GLP-1 medications continue taking the costly drugs anyway. This highlights a significant cost-management challenge for self-funded employers covering obesity treatments without strict utilization management or stopping rules. Plan sponsors must implement tighter clinical oversight and outcomes-based management to prevent sustained spending on ineffective specialty therapies.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Managed Healthcare Executive</t>
+          <t>Insurance Business</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:32:25 GMT</t>
+          <t>Wed, 14 Oct 2026 11:46:38 GMT</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPYTA3dnRyM1VEb1ZYWjlqVUV3WncxSDRrUll5bzVFeElEeDBRNWVZM0NaLXpaUUpESzJDeHBIUGRNMnZSRnRncGxldGd6Q3ZIUUdHOVh6SFVmUlBnOFh0cEJCQmc4THIwZ0dRWjh6WGtnMEVfRGkxTk1WY25YOG1GVWRuWC1EVmZ2QkpJZUIyN2VkX2JQZlBMdk5GM1dTR01zRWVGYXRmTmdBZ2pKeFd4N2JhTHZKcGJPR3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizgFBVV95cUxPRWRpajE5OUpQYzFXRTJOTjVSc2xJT3BBaGp1LUVjLUFWX2lTZkx1OFZldnhrOTlkY21DMWhEOFR5dDVwTFhReWotdlFlLTBGdGZHTnMtMW1pNmI4VEJ1dDEzSjdNdDh6cnBpQnRPNnNfWDlzMlkyRjluNnJmSFRpODBLSmMzVDFuVGpCOTFtV3ZpVmcwUTZzbVpyZ0FUUUZQSXZUNVhwWG16aHJrc0Npb29BU2tnZ242RWtQQ1lsOHdkd2JqYkJ3WmhlbHRKZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -537,27 +537,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Employer-Sponsored Healthcare Cost Growth Driven Primarily by Price Increases</t>
+          <t>Federal Agencies Finalize Transparency in Coverage Rules for Health Plans</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Recent analysis highlights that rising healthcare costs for U.S. employers are primarily driven by underlying price increases rather than utilization shifts. For self-funded plan sponsors, this underscores the critical need for aggressive pharmacy and medical cost containment strategies to combat inflationary pressures.</t>
+          <t>Federal departments have finalized new Transparency in Coverage rules, impacting health plans and issuers regarding public reporting requirements. This regulatory update directly affects self-funded employers and PBMs by establishing stricter compliance and data disclosure mandates for health plan pricing.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Managed Healthcare Executive</t>
+          <t>JD Supra</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:41:15 GMT</t>
+          <t>Wed, 14 Oct 2026 20:40:08 GMT</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxQMTdFSzhrSi1uMEhENF9lTjVMX0Ewb2dsUE9sdGNpNTlFYlM5Q2pOZ2tyb2xKdnlrdnI1aXJPVTVBeGdTR1o1enZ2a3VuSUZBSDdDbjVDbFl0SE4yQ2UxTjQwb0JzekZ6ZlBZVExYZlZ6MUxOZkx1b192blpXVng2d2F1YjhmbEtjc1hHX041eExFb2lsekROaTVwWDNIOFExWTZJU0RWOHZoaHM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPRTdvYXFxWDRKNFItQm8yS3NnR0lTczJEajFBYjRfeGs1Wm4zaEhmRGlWeTJRN2xTZDVpa1ZVOWU1bi0tQUlZQXZ6dnQ0ZDVGWUhZcDBYaEJrUzFNRjFEdUp2ZkNiZHhJZG5lcDN5N2VFYmRDaDJ0cXVjcXl0WWd2c2dQT1JCZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -567,27 +567,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>U.S. Hospitals Sue Over Revised 340B Rebate Models</t>
+          <t>Celltrion Nears Major US PBM Formulary Deals for Biosimilars Ahead of Q4</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Hospital groups are challenging revised 340B drug manufacturer rebate and pricing models in federal court. This ongoing legal battle impacts the broader drug supply chain, contract pharmacy arrangements, and drug cost dynamics that affect employer-sponsored health plans.</t>
+          <t>Celltrion is closing in on major US PBM formulary negotiations with anticipated contract signings in the fourth quarter. This development directly impacts self-funded employers by potentially expanding biosimilar market access, driving competition, and creating new opportunities to lower specialty drug costs.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>NAVLIN DAILY</t>
+          <t>BigGo Finance</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 08:10:12 GMT</t>
+          <t>Wed, 14 Oct 2026 02:26:00 GMT</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxNQWowNEczMFF1VmNYV190THhHZ0hRQXNZd3JGM05zNEhKeklCLWZTeXBVemRtM0FzdHl6VjBUYkVWbG0zWWFSazR4LVZDNnVUTDc1dTNRd1d5WlpSejJUMWVHYnR1MGY2T2tBOVFTbTdMNW1VUlNQMXNzTUF4Z295eF8zaTI4dzdVSW9YcE5XeS1tZy1aVkxYc1VaOFBMLTZYRXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE8zOU91Y2FLQ0hDT2Rnenh6YWNHOEpGbGw1T0duZHlHc2R1a0VKdXdLNUhLcGhlMGF4Z2hyb3Z2bFFjVjdDQktZa3dxdGNPT3FzSlVkVlhSNWhMMnNJSkt2dEhBQ09yeUtfWlVTWnJqbmQ5TXlaOHc?oc=5</t>
         </is>
       </c>
     </row>
@@ -597,27 +597,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>UCSF Study Links PBM Rebates to Opioid Manufacturers, Sparking Reform Calls</t>
+          <t>Pennsylvania AG Sues Over Alleged Insulin Price Manipulation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Researchers at UCSF have uncovered undisclosed financial ties between pharmacy benefit managers and opioid manufacturers tied to drug rebate structures. The findings add momentum to legislative efforts targeting PBM transparency and rebate practices, directly impacting self-funded employers seeking greater accountability in drug spend.</t>
+          <t>The Pennsylvania Attorney General has filed a lawsuit alleging collusion to artificially inflate insulin prices. This legal action highlights ongoing state-level scrutiny and antitrust concerns regarding drug pricing practices, which directly impact self-funded employers managing high-cost specialty medications like insulin.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Medical Daily</t>
+          <t>Yahoo</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 23:22:52 GMT</t>
+          <t>Wed, 14 Oct 2026 13:35:38 GMT</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOU1F3RWhSUEF1X1VxVU9BdmNCVnB0V1dWcjR1c3F0RklTMzZnTHhrRDBtV2Y1SDdlc3RRZEJQX0NZckNaRzBSbllaejk2aDF0SHVMMWo0QXVmN2FVT1N2bGFfUTA3WkhHRkt6T3hxaWFEdkxzNWlsQUJmSzJRTG9lRTAzLTN4OWhKb3oxem5fV3ljOHM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxPNGF6YURINmtObDJWM2dwWk9VZTBKcU56M3ctQTdjOHVHU0Q0R1hyN0hLX3FiMkNiamUxT3BDX25jeFFfeHNvZUhhZzdHVVpNOHJqY3ZiYnN6Rk5WNWV1U19JTzU0SkNhMmNlVC1INjVNSUlPYkxjQlZWdXdrTERPX3JvYU5NanEzekFDQ2ZfS205SFdmT1hJ?oc=5</t>
         </is>
       </c>
     </row>
@@ -627,207 +627,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Employer Health Plan Costs Projected to Rise 8.2% Amid Data Lags</t>
+          <t>State Sues Insulin Manufacturers and PBMs Over Artificial Price Increases</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Projected employer health plan costs are expected to climb 8.2%, driven by underlying cost pressures and delayed claims data visibility. This rising trend directly impacts self-funded employers seeking proactive pharmacy benefit management strategies to control escalating health benefit expenditures.</t>
+          <t>A state attorney general has filed a lawsuit against major insulin manufacturers and pharmacy benefit managers, alleging collusion to artificially inflate drug prices. This litigation increases legal and regulatory scrutiny on PBM pricing models and rebate practices, carrying significant implications for self-funded employers seeking transparent drug costs.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Human Resources Director</t>
+          <t>Northeast Times</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 23:35:10 GMT</t>
+          <t>Wed, 14 Oct 2026 13:38:43 GMT</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOWjdMVGJzdXB5SDdXczFRbE5jUW9KR01ta25jakllckc5YjcyOXFFQW55WUIyU2dQRDVHSTFzc19pNVpYTFNoSnV4LUxvb1NBNTh5OUhtc2pKUENPbGc2ZUM2OHZJb3Q4ZUVLVy1jaFU3cnBrMHFOeXJsaU9iSFg2MFpKZWhTdGoyUjZxNTBwaGV6MzB1OXNUT2VRcnVUcmpRZWppSkRQb3YwYXRmUVZwd05TbDM?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Walmart Expands Zero-Cost Coverage for Insulin and GLP-1s for Employees</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Walmart is offering certain GLP-1 medications and insulin at zero cost to its employees as part of its health plan benefits. This move highlights how major self-funded employers are strategically managing chronic conditions and wrestling with the surging costs of obesity drugs. For self-funded employers and PBMs, it underscores the ongoing competitive pressure to balance benefit generosity with escalating specialty drug spend.</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Bloomberg.com</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 13:30:00 GMT</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNSV9IZUdFdUtxNUxXbER5eUtvZlVkeFN4Sll4TlNMdHYzVWZfRlFuM0xPRjh1V1h0Q05xSHpKVkVtMExSN2hLNkJnczMyN1pENlkzdlpiYlZJVUdYVy1zTFFnMWx3U3I2VUFKWFhJaXh3dVoxSkJJeGUxdm1HbEw5MUkyM3JEelR0ZEFVM0RBQ0NNRzdvU2gwZ1hhcURvSEs2Q29BYjdTN3Znd20wS2ZV?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Walmart Expands Employee Health Benefits to Cover GLP-1s and Insulin at No Cost</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Walmart is updating its employer-sponsored health plan to provide zero-cost coverage for GLP-1 weight-loss medications, insulin, and inhalers. This move highlights major self-funded employers aggressively tackling chronic disease and obesity costs despite escalating utilization pressures. For self-funded plans and PBMs, it underscores the ongoing strategic debate around managing high-cost specialty drugs versus long-term health outcomes.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>CNBC</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 17:07:19 GMT</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxPWXotQk5KcGxxckYzSjJhdkhsX2pMbXZJUlR1djg2Qk5OUXF1UUZxTTZuWVFHUXJaZTk0ZnlKUHhlOTIzOTdkTDhaSmYxSGFtMlVQTU95RUxOa3lCcTlGYmdqUlAtcDVvX044TTR6U2dUNDduOERzYjZmYXZITEo4RThQWGxWMGVTWVcwdWhCUdIBlAFBVV95cUxOUmwxWGtjSGV6aDR2NElVeF8tZEJ1SU1iSW9mdjJPRGpSN0NUSXluU05SZk1XYWhJalRBanRGejZ0d0FWdjVfbFZiallXcElobjlIeEdYUUE3ZUY0WmRaTWVyellpQWRsZlRoV29kbDY5TGlJRkpzOXFaTU9mVlp4b3VDQW9pS3VhOExQTUc5ZEpjVm5L?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Formycon Files US Biosimilar for Keytruda</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Formycon has submitted a US regulatory filing for a Keytruda biosimilar, representing a major milestone in oncology cost management. As high-cost specialty biologics face patent expirations, upcoming biosimilars offer self-funded employers significant opportunities to lower net specialty drug spend. PBMs will need to strategically update their formulary positioning and utilization management to drive adoption of these lower-cost alternatives.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>insights.citeline.com</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 10:44:32 GMT</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMijAJBVV95cUxNYmxWSV83UUlxcVhvRGFQT1JfcUp0d1RPYW5la19ORXlsOWgySVpFdmU1Ym5EOTV5Z0Y1R2lydklWMHl4NFUxei14VUNFQ2RwR1V0b2g0RWZaRlF6U0p5WVZoV190eXRGY1RscEJrYV83WDJ5YnVEMnBlZ1R5RkFXZG45OVhVcDZ6SkdQWDVMUk5xNmYyaEUzSUxXb09CRU1uMjhJakkwV3dGQ19RVVNpcWZ2Yk9rRFdydThabUZzQmRKT0tscmVtbklIUE44UzlYd3htMk5HTE5QcC1NQzU0RWJXN05UMHl4T19LZDB6VGZZVERkaW01VWlBZW9yT2RkS0FTNms2TEl4VjF0?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Walmart Expands Zero-Cost Drug Benefit for Eligible Employees</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Walmart is introducing a benefit covering over 250 medications at zero cost for eligible employees, signaling a continued shift toward value-based plan design and chronic condition management. For self-funded employers and PBMs, this highlights innovative benefit strategies aimed at improving medication adherence and managing overall health plan spend.</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Yahoo Finance</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 14:35:38 GMT</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxOQzRkcDk4NWNFdjdBQmpCWUFxTjE2SkNVS2tQbWh2cTdHSGZ5YkptNlFaUFJ1dVVFZlFIUEY3b3JCZVhaRXQ2TVduVFgycnl4Um1pQzZQNjI3RWpwRE4xN2xzazlMckF5ZklFWmM5LWJIU2RnUzFRT3R3T0xPQ2huUm5STFRrakNhZnFXakx6LUtMajA?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Walmart to Provide Free GLP-1s and Insulin to Employees by 2027</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Walmart announced plans to offer zero-copay coverage for popular diabetes and weight-loss drugs like Ozempic and Mounjaro, as well as insulin, to its U.S. employees starting in 2027. This landmark self-funded employer benefit move will put immense pressure on other large corporations to evaluate their own specialty drug coverage and cost-sharing strategies for GLP-1s.</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>BigGo Finance</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 18:29:00 GMT</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTFBEcXVzTTRuVGZTU0RkZ2VqOVc2ZDd4aTNpQ0tJSGRyZ1ZlemFpUVlTLXNNZ3Q0am9MR25hVzJla2hOZjFPMFd6d2x2YllOT3JCMFIwX2ZyaHdvM1dLWl9OZzZtcF91X0swYVA4SjNrZXNEdnBsc0E?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>UnitedHealth Initiatives Focus on Prior Authorization and Pharmacy Transparency</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Truist reports that UnitedHealth is advancing initiatives centered on prior authorizations and pharmacy transparency. This is significant for self-funded employers and PBMs navigating increasing regulatory scrutiny and employer demand for greater visibility into drug benefit operations.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>marketscreener.com</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 18:52:23 GMT</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi5AFBVV95cUxNcU9CS2t4bTdBeWJtRVhVSWVBTnFSLXN2TEVoSUlWRVhXdFUzSGxLX3YwSTN0TEkzZXRhbnkzTWlBVHMtZ1dTb0JQenlINkJqdlJxd1ppa3NnOG9NTDBmREFKQ0wxaU1QZldPdHN1b0VfcGM5Y05DNV9tbUx1NXpvZ2VIRXZaeWRtQTQtbVFVTU1FY2VPcU15bmJJaHZLdWxaMV9yTkNFbjdPYjA3aXFiT3habnkxbkdNbl9famZmN1NOWW8xbjNBaUVPcjU0UUJQTGthSm81QktuRW1oeWNuWFV2cUI?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxPUGFSRUwxU3RweWFjNkFPZnRpbW15N1REcGpJVEpWZTNaUDJKeUhuZ2NBVzk0VEhLTUJCN3JkNzkwQnhHSjVDRFQ4WEpDbHlxbUZFeXEzb2JuLVdNNnNFTk0tejI4a3hoRW1DbDg1cnFiVk5ZNG1ldjlpdG8tcXFReFpsQ1JLT2JlV0lwWnczTTh3Qlo3QkRRY3NzQ01TQXNaTDFiTjREYkF2SzhlZ2l1RXV5eUxxdw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>